<commit_message>
Refine OG0021 quiz v2 question design
</commit_message>
<xml_diff>
--- a/v2/OG0021/OG0021_ReadingQuiz.xlsx
+++ b/v2/OG0021/OG0021_ReadingQuiz.xlsx
@@ -88,7 +88,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
     <fill>
@@ -103,7 +103,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,12 +155,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -170,13 +164,16 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -185,7 +182,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -638,7 +638,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Setting Builder</t>
+          <t>Setting Image Choice</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -648,17 +648,17 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Build the story setting.</t>
+          <t>Where does Milo go to look for his color?</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>label cards</t>
+          <t>SC01/03/06/10 images</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>who=Milo / where=home / situation=has colors</t>
+          <t>Option B</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -671,7 +671,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Component Weight</t>
+          <t>Weighted MCQ</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Look at the scene. Build what Milo does.</t>
+          <t>Put the story words in order.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Milo looks for his lost color.</t>
+          <t>Milo walks into the forest.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -798,7 +798,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>How does Milo react in this scene?</t>
+          <t>How does Milo feel here?</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Thought Bubble</t>
+          <t>Internal Response MCQ</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Put Milo's thought in the bubble.</t>
+          <t>What is Milo thinking?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Weighted Thought Card</t>
+          <t>Weighted MCQ</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Cause→Result Chain</t>
+          <t>Ending Scene Sequence</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -898,17 +898,17 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Make the cause and result chain.</t>
+          <t>Put the ending scenes in order.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>text cards</t>
+          <t>SC06/07/08/09 images</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>cry → colors come back</t>
+          <t>SC06 → SC07 → SC08 → SC09</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Component Weight</t>
+          <t>Weighted Position</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Q01</t>
         </is>
@@ -1107,7 +1107,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Q02</t>
         </is>
@@ -1149,7 +1149,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Q03</t>
         </is>
@@ -1191,7 +1191,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Q04</t>
         </is>
@@ -1233,7 +1233,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Q05</t>
         </is>
@@ -1275,7 +1275,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Q06</t>
         </is>
@@ -1317,7 +1317,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Q07</t>
         </is>
@@ -1372,16 +1372,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
@@ -1389,51 +1389,51 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q01 — Setting Builder | Story Grammar: Setting</t>
+          <t>Q01 — Setting Image Choice | Story Grammar: Setting</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Build the story setting by placing cards into Who / Where / At first slots.</t>
+          <t>Question: Where does Milo go to look for his color?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Slot</t>
+          <t>Option</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Correct Card</t>
+          <t>Scene / Resource</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>Correct?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>SG Role</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Slot Weight</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Near-Miss Examples</t>
-        </is>
-      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Weight Rationale</t>
+          <t>Distractor Rationale</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Max Points</t>
+          <t>Student Weakness Signal</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1450,86 +1450,88 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Who</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Milo</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC01_I</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Character in setting</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>butterfly</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Identifies the story focus before the problem begins.</t>
-        </is>
-      </c>
-      <c r="G5" s="6">
-        <f>D5/SUM($D$5:$D$7)*100</f>
-        <v/>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>setting_actor_confusion</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
+        <v>35</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Opening character</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>인물 소개 장면과 실제 탐색 장소를 혼동함</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Opening/setting detail confusion</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>setting_actor_scene</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>his colorful home</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Place / initial world</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>blue pond</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Separates opening place from later consequence scene.</t>
-        </is>
-      </c>
-      <c r="G6" s="4">
-        <f>D6/SUM($D$5:$D$7)*100</f>
-        <v/>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>setting_place_shift</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC03_I</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Place setting</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Milo walks into the forest.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>correct_setting_place</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
@@ -1538,66 +1540,105 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>At first</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>has many colors</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC06_I</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Initial situation</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>lost color</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Distinguishes normal beginning from initiating event.</t>
-        </is>
-      </c>
-      <c r="G7" s="6">
-        <f>D7/SUM($D$5:$D$7)*100</f>
-        <v/>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>initial_state_problem_confusion</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
+        <v>55</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Later place</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>중요 장소인 연못을 탐색이 시작된 장소와 혼동함</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Later consequence place confusion</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>setting_later_place</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D8" s="7">
-        <f>SUM(D5:D7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="7">
-        <f>SUM(G5:G7)</f>
-        <v/>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC10_I</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Ending place</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>결말의 집 장면을 주요 탐색 장소로 혼동함</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Ending/opening place confusion</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>setting_ending_place</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_v2_q01_setting" | result.sg_element="setting" | result.score_raw=&lt;pts&gt;</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A11:I11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1638,7 +1679,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Resource: Audio/OG0021_SC02_ST01_N_A.mp3</t>
         </is>
@@ -1692,7 +1733,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1702,12 +1743,12 @@
           <t>OG0021_SC02_I</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1737,7 +1778,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1747,12 +1788,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1782,7 +1823,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1792,12 +1833,12 @@
           <t>OG0021_SC06_I</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="6" t="n">
         <v>30</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1827,7 +1868,7 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -1837,12 +1878,12 @@
           <t>OG0021_SC09_I</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1872,7 +1913,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q02_init_event" | result.sg_element="initiating_event" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -1919,21 +1960,21 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Look at SC03. Build what Milo does.</t>
+          <t>Question: Put the story words in order.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Correct sentence: "Milo looks for his lost color."</t>
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Correct sentence from SC03_ST01_N: "Milo walks into the forest."</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Scrambled words: looks | color. | his | Milo | lost | for</t>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Scrambled words: walks | forest. | Milo | the | into</t>
         </is>
       </c>
     </row>
@@ -1975,20 +2016,20 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Milo</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="13" t="n">
         <v>1.5</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1996,7 +2037,7 @@
           <t>Identifies actor of attempt.</t>
         </is>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="14">
         <f>D7/SUM($D$7:$D$12)*100</f>
         <v/>
       </c>
@@ -2007,20 +2048,20 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>looks</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>walks</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Action verb</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="13" t="n">
         <v>2.5</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2028,8 +2069,8 @@
           <t>Core attempt action; highest weight.</t>
         </is>
       </c>
-      <c r="F8" s="15">
-        <f>D8/SUM($D$7:$D$12)*100</f>
+      <c r="F8" s="14">
+        <f>D8/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -2039,52 +2080,52 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>for</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>into</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Preposition</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="n">
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Direction word</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n">
         <v>1.5</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Links action to goal.</t>
-        </is>
-      </c>
-      <c r="F9" s="15">
-        <f>D9/SUM($D$7:$D$12)*100</f>
+          <t>Connects action to place.</t>
+        </is>
+      </c>
+      <c r="F9" s="14">
+        <f>D9/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>goal_link</t>
+          <t>direction_word</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>his</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="n">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>the</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Possessive</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="n">
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -2092,92 +2133,60 @@
           <t>Small syntax support.</t>
         </is>
       </c>
-      <c r="F10" s="15">
-        <f>D10/SUM($D$7:$D$12)*100</f>
+      <c r="F10" s="14">
+        <f>D10/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>possessive</t>
+          <t>article</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>lost</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>forest.</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Goal state</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>2</v>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Place noun</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>2.5</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Shows the problem he is trying to solve.</t>
-        </is>
-      </c>
-      <c r="F11" s="15">
-        <f>D11/SUM($D$7:$D$12)*100</f>
+          <t>Shows where the attempt begins.</t>
+        </is>
+      </c>
+      <c r="F11" s="14">
+        <f>D11/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>problem_state</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>color.</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Goal noun</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Core goal of the attempt.</t>
-        </is>
+          <t>attempt_place</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D12" s="15">
+        <f>SUM(D7:D11)</f>
+        <v/>
       </c>
       <c r="F12" s="15">
-        <f>D12/SUM($D$7:$D$12)*100</f>
-        <v/>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>attempt_goal</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D13" s="7">
-        <f>SUM(D7:D12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="7">
-        <f>SUM(F7:F12)</f>
+        <f>SUM(F7:F11)</f>
         <v/>
       </c>
     </row>
@@ -2213,7 +2222,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Milo looks for his lost color.</t>
+          <t>Milo walks into the forest.</t>
         </is>
       </c>
       <c r="B17" s="17" t="n">
@@ -2221,7 +2230,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Attempt action and goal fully understood.</t>
+          <t>Exact story sentence restored.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -2233,10 +2242,10 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Milo looks for lost his color.</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="n">
+          <t>Milo walks the into forest.</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
         <v>83</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -2246,22 +2255,22 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>possessive placement</t>
+          <t>function word placement</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Milo color. lost his for looks</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="n">
-        <v>14</v>
+          <t>forest. into the walks Milo</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>17</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Goal words known but action chain is broken.</t>
+          <t>Place is known but action sequence is broken.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2312,12 +2321,12 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: How does Milo react in this scene?</t>
+          <t>Question: How does Milo feel here?</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -2371,7 +2380,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -2381,12 +2390,12 @@
           <t>Happy</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2416,7 +2425,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2426,12 +2435,12 @@
           <t>Sad</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2461,7 +2470,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2471,12 +2480,12 @@
           <t>Angry</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="6" t="n">
         <v>40</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2506,7 +2515,7 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -2516,12 +2525,12 @@
           <t>Surprised</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -2551,7 +2560,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q04_reaction" | result.sg_element="reaction" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -2591,19 +2600,19 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q05 — Thought Bubble | Story Grammar: Internal Response</t>
+          <t>Q05 — Internal Response MCQ | Story Grammar: Internal Response</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Put Milo's thought in the bubble.</t>
+          <t>Question: What is Milo thinking?</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -2657,22 +2666,22 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Everyone has a color but me.</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+          <t>Everyone has their own color.</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2687,7 +2696,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Captures Milo's inner comparison and loneliness.</t>
+          <t>Uses the actual SC06 thought/sentence to infer Milo's inner state.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2702,22 +2711,22 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>I want to play with butterflies.</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
+          <t>I want to fly with the butterfly.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2727,7 +2736,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Confuses action context with inner thought.</t>
+          <t>Confuses earlier butterfly scene with Milo's thought.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -2742,37 +2751,37 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>I am the fastest chameleon.</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
+          <t>The pond is very blue.</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="12" t="n">
-        <v>0</v>
+      <c r="D8" s="6" t="n">
+        <v>45</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Unrelated self-belief</t>
+          <t>Surface observation</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Opposite of the vulnerable internal state.</t>
+          <t>Sees visual detail but not internal state.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Guessing / no inference</t>
+          <t>Surface-level inference</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -2789,7 +2798,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>The pond is very blue.</t>
+          <t>I do not need my color.</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -2798,21 +2807,21 @@
         </is>
       </c>
       <c r="D9" s="11" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Surface observation</t>
+          <t>Opposite motive</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Sees visual detail but not internal state.</t>
+          <t>Contradicts Milo's motivation to find his color.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Surface-level inference</t>
+          <t>Motive inversion</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -2822,7 +2831,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q05_internal" | result.sg_element="internal_response" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -2845,12 +2854,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
@@ -2861,41 +2870,41 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q06 — Cause→Result Chain | Story Grammar: Consequence</t>
+          <t>Q06 — Ending Scene Sequence | Story Grammar: Consequence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Make the cause and result chain.</t>
+          <t>Question: Put the ending scenes in order.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Slot</t>
+          <t>Scene</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Correct Card</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Slot Weight</t>
+          <t>Correct Pos</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Max Points</t>
+          <t>Scene Weight</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Distractors</t>
+          <t>SG Role</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -2915,39 +2924,38 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Cause</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Milo cries by the pond.</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="D5" s="6">
-        <f>C5/SUM($C$5:$C$6)*100</f>
-        <v/>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>The butterfly turns gray.</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Identifies the action/event that triggers the result.</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>wrong_cause</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>SC06</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>OG0021_SC06_I</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Cause / low point</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Milo cries; this begins the ending chain.</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>missed_cause_scene</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>consequence</t>
         </is>
@@ -2956,34 +2964,33 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>SC07</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>His colors come back.</t>
+          <t>OG0021_SC07_I</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="D6" s="4">
-        <f>C6/SUM($C$5:$C$6)*100</f>
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1.5</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Milo stays gray forever.</t>
+          <t>Immediate result</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Result is the core consequence and receives slightly higher weight.</t>
+          <t>The pond shines after the tear falls.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>wrong_result</t>
+          <t>immediate_result_shift</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -2993,17 +3000,89 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SC08</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>OG0021_SC08_I</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Internal turn</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Milo realizes his color may be inside him.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>realization_order</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>consequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>SC09</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>OG0021_SC09_I</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Final consequence</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Milo's colors come back; final outcome receives high weight.</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>final_result_order</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>consequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C7" s="7">
-        <f>SUM(C5:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="7">
-        <f>SUM(D5:D6)</f>
+      <c r="D9" s="15">
+        <f>SUM(D5:D8)</f>
         <v/>
       </c>
     </row>
@@ -3098,7 +3177,7 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3108,12 +3187,12 @@
           <t>Colors keep you safe.</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="8" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3143,7 +3222,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3153,12 +3232,12 @@
           <t>Friends always help you.</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="6" t="n">
         <v>30</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3188,7 +3267,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3198,12 +3277,12 @@
           <t>Your color is inside you.</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3233,7 +3312,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3243,12 +3322,12 @@
           <t>The world has many colors.</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3278,7 +3357,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q07_synthesis" | result.sg_element="synthesis" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -3357,7 +3436,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
@@ -3374,12 +3453,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>component weighted score</t>
+          <t>weighted option score</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Understands initial time/place/situation.</t>
+          <t>Understands the key place/background for the story action.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -3394,7 +3473,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Initiating Event</t>
         </is>
@@ -3431,7 +3510,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Attempt</t>
         </is>
@@ -3468,7 +3547,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Reaction</t>
         </is>
@@ -3505,7 +3584,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Internal Response</t>
         </is>
@@ -3522,7 +3601,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>thought-card score</t>
+          <t>option score</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3542,7 +3621,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Consequence</t>
         </is>
@@ -3559,7 +3638,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>cause/result component score</t>
+          <t>weighted scene position</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3579,7 +3658,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Synthesis</t>
         </is>
@@ -3616,7 +3695,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Overall Reading Score = average(6 Story Grammar axes) × 0.8 + Synthesis × 0.2</t>
         </is>

</xml_diff>

<commit_message>
Refine OG0021 v2 story-flow quiz
</commit_message>
<xml_diff>
--- a/v2/OG0021/OG0021_ReadingQuiz.xlsx
+++ b/v2/OG0021/OG0021_ReadingQuiz.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUIZ_LIST" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q01_SETTING" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q01_CONSEQUENCE" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q02_INIT_EVENT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q03_ATTEMPT" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q04_REACTION" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q05_INTERNAL" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q06_CONSEQUENCE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q06_SETTING" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q07_SYNTHESIS" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SG_SCORING" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LRS_MAPPING" sheetId="10" state="visible" r:id="rId10"/>
@@ -88,7 +88,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -103,7 +103,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,6 +155,15 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -164,16 +173,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,10 +185,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -560,21 +560,21 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OG0021 Reading Quiz v2 — Story Grammar + Synthesis</t>
+          <t>OG0021 Reading Quiz v2 - Story Grammar + Synthesis</t>
         </is>
       </c>
     </row>
@@ -638,27 +638,27 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Setting Image Choice</t>
+          <t>Story Scene Sequence</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Consequence</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Where does Milo go to look for his color?</t>
+          <t>Put the story scenes in order.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>SC01/03/06/10 images</t>
+          <t>SC01/02/03/06/09 images</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Option B</t>
+          <t>SC01 -&gt; SC02 -&gt; SC03 -&gt; SC06 -&gt; SC09</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -666,17 +666,17 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>consequence</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Weighted MCQ</t>
+          <t>Weighted Position</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Q01_SETTING</t>
+          <t>Q01_CONSEQUENCE</t>
         </is>
       </c>
     </row>
@@ -888,27 +888,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ending Scene Sequence</t>
+          <t>Setting MCQ</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Consequence</t>
+          <t>Setting</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Put the ending scenes in order.</t>
+          <t>Who is Milo at the beginning?</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>SC06/07/08/09 images</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>SC06 → SC07 → SC08 → SC09</t>
+          <t>Option B</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
@@ -916,17 +916,17 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>consequence</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Weighted Position</t>
+          <t>Weighted MCQ</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Q06_CONSEQUENCE</t>
+          <t>Q06_SETTING</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>v2 keeps one primary Story Grammar element per scored question. Q7 Synthesis is reported separately from the six-axis graph.</t>
+          <t>v2 uses story-flow question order while keeping one primary Story Grammar score per Q01-Q06. Q07 Synthesis is reported separately and contributes to the overall score.</t>
         </is>
       </c>
     </row>
@@ -1007,18 +1007,18 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LRS xAPI Mapping — OG0021 v2</t>
+          <t>LRS xAPI Mapping - OG0021 v2</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Q01</t>
         </is>
@@ -1077,247 +1077,247 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>quiz_OG0021_v2_Q01_setting</t>
+          <t>quiz_OG0021_v2_Q01_consequence</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>consequence</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>scene_order, component_scores</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Consequence gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Q02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q02_initiating_event</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>true/false</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>option_selected, audio_src</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Initiating event gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q03_attempt</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>attempt</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>word_order, word_scores</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Attempt/action gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q04_reaction</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>true/false</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>option_selected</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Reaction/emotion gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q05_internal_response</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>internal_response</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>true/false</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>option_selected</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Inference gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q06_setting</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
           <t>setting</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>slot_values, component_scores</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>true/false</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>option_selected</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Setting gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Q02</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q02_initiating_event</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>initiating_event</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>true/false</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>option_selected, audio_src</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Initiating event gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q03_attempt</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>attempt</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>word_order, word_scores</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Attempt/action gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q04_reaction</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>true/false</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>option_selected</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Reaction/emotion gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q05_internal_response</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>internal_response</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>true/false</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>thought_selected</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Inference gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Q06</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q06_consequence</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>cause_card,result_card</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Consequence gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Q07</t>
         </is>
@@ -1372,53 +1372,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q01 — Setting Image Choice | Story Grammar: Setting</t>
+          <t>Q01 - Story Scene Sequence | Story Grammar: Consequence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Where does Milo go to look for his color?</t>
+          <t>Question: Put the story scenes in order.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Scene</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Scene / Resource</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Correct?</t>
+          <t>Correct Pos</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Score</t>
+          <t>Scene Weight</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1428,217 +1427,233 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Distractor Rationale</t>
+          <t>Weight Rationale</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Student Weakness Signal</t>
+          <t>Error Tag</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Error Tag</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
           <t>LRS</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>SC01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>OG0021_SC01_I</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Opening character</t>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Opening state</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>인물 소개 장면과 실제 탐색 장소를 혼동함</t>
+          <t>Shows Milo before the problem begins; useful context but lower weight than problem/result.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Opening/setting detail confusion</t>
+          <t>missed_opening_state</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>setting_actor_scene</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
+          <t>consequence</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SC02</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OG0021_SC02_I</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Problem begins</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Milo wakes up gray; this is the key event that drives the rest of the story.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>missed_problem_start</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SC03</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Place setting</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Milo walks into the forest.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>correct_setting_place</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Attempt begins</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Milo starts searching in the forest; a middle bridge scene.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>attempt_position_shift</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>attempt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>SC06</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>OG0021_SC06_I</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Later place</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>중요 장소인 연못을 탐색이 시작된 장소와 혼동함</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Later consequence place confusion</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>setting_later_place</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>OG0021_SC10_I</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Ending place</t>
+      <c r="C8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Low point / reaction</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>결말의 집 장면을 주요 탐색 장소로 혼동함</t>
+          <t>Milo cries by the pond; shows the consequence before recovery.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Ending/opening place confusion</t>
+          <t>reaction_position_shift</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>setting_ending_place</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_v2_q01_setting" | result.sg_element="setting" | result.score_raw=&lt;pts&gt;</t>
+          <t>reaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>SC09</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>OG0021_SC09_I</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Final result</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Milo's colors come back; final consequence gets high weight.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>missed_final_result</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>consequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D10" s="7">
+        <f>SUM(D5:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q01_consequence" | result.sg_element="consequence" | result.score_raw=&lt;pts&gt;</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1667,7 +1682,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q02 — Listening Scene Match | Story Grammar: Initiating Event</t>
+          <t>Q02 - Listening Scene Match | Story Grammar: Initiating Event</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1694,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Resource: Audio/OG0021_SC02_ST01_N_A.mp3</t>
         </is>
@@ -1733,7 +1748,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1743,12 +1758,12 @@
           <t>OG0021_SC02_I</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1778,7 +1793,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1788,12 +1803,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1823,7 +1838,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1833,12 +1848,12 @@
           <t>OG0021_SC06_I</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="12" t="n">
         <v>30</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1868,7 +1883,7 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -1878,12 +1893,12 @@
           <t>OG0021_SC09_I</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="13" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1913,7 +1928,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q02_init_event" | result.sg_element="initiating_event" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -1953,7 +1968,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q03 — Scene-Anchored Unscramble | Story Grammar: Attempt</t>
+          <t>Q03 - Scene-Anchored Unscramble | Story Grammar: Attempt</t>
         </is>
       </c>
     </row>
@@ -1965,14 +1980,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Correct sentence from SC03_ST01_N: "Milo walks into the forest."</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Scrambled words: walks | forest. | Milo | the | into</t>
         </is>
@@ -2016,20 +2031,20 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Milo</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2037,8 +2052,8 @@
           <t>Identifies actor of attempt.</t>
         </is>
       </c>
-      <c r="F7" s="14">
-        <f>D7/SUM($D$7:$D$12)*100</f>
+      <c r="F7" s="15">
+        <f>D7/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -2048,20 +2063,20 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>walks</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Action verb</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>2.5</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2069,7 +2084,7 @@
           <t>Core attempt action; highest weight.</t>
         </is>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="15">
         <f>D8/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
@@ -2080,20 +2095,20 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>into</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Direction word</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>1.5</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -2101,7 +2116,7 @@
           <t>Connects action to place.</t>
         </is>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="15">
         <f>D9/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
@@ -2112,20 +2127,20 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>the</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -2133,7 +2148,7 @@
           <t>Small syntax support.</t>
         </is>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="15">
         <f>D10/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
@@ -2144,20 +2159,20 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>forest.</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Place noun</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>2.5</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -2165,7 +2180,7 @@
           <t>Shows where the attempt begins.</t>
         </is>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="15">
         <f>D11/SUM($D$7:$D$11)*100</f>
         <v/>
       </c>
@@ -2176,16 +2191,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="7">
         <f>SUM(D7:D11)</f>
         <v/>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="7">
         <f>SUM(F7:F11)</f>
         <v/>
       </c>
@@ -2193,7 +2208,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SECTION B — Partial Score Examples</t>
+          <t>SECTION B - Partial Score Examples</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2260,7 @@
           <t>Milo walks the into forest.</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="12" t="n">
         <v>83</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -2265,7 +2280,7 @@
           <t>forest. into the walks Milo</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="11" t="n">
         <v>17</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2314,7 +2329,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q04 — Feeling Match | Story Grammar: Reaction</t>
+          <t>Q04 - Feeling Match | Story Grammar: Reaction</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2341,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -2380,7 +2395,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -2390,12 +2405,12 @@
           <t>Happy</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="13" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2425,7 +2440,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2435,12 +2450,12 @@
           <t>Sad</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2470,7 +2485,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2480,12 +2495,12 @@
           <t>Angry</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="12" t="n">
         <v>40</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2515,7 +2530,7 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -2525,12 +2540,12 @@
           <t>Surprised</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -2560,7 +2575,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q04_reaction" | result.sg_element="reaction" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -2600,7 +2615,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q05 — Internal Response MCQ | Story Grammar: Internal Response</t>
+          <t>Q05 - Internal Response MCQ | Story Grammar: Internal Response</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2627,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -2666,7 +2681,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -2676,12 +2691,12 @@
           <t>Everyone has their own color.</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2711,7 +2726,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2721,12 +2736,12 @@
           <t>I want to fly with the butterfly.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2736,22 +2751,27 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
+          <t>Earlier action</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
           <t>Confuses earlier butterfly scene with Milo's thought.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Thought/action confusion</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>attempt</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2761,12 +2781,12 @@
           <t>The pond is very blue.</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="12" t="n">
         <v>45</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2776,22 +2796,27 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
+          <t>Visual detail</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
           <t>Sees visual detail but not internal state.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Surface-level inference</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>internal_response</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -2801,12 +2826,12 @@
           <t>I do not need my color.</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="13" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -2816,22 +2841,27 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
+          <t>Contradiction</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
           <t>Contradicts Milo's motivation to find his color.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Motive inversion</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>internal_response</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q05_internal" | result.sg_element="internal_response" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -2854,242 +2884,273 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q06 — Ending Scene Sequence | Story Grammar: Consequence</t>
+          <t>Q06 - Setting MCQ | Story Grammar: Setting</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Put the ending scenes in order.</t>
+          <t>Question: Who is Milo at the beginning?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Scene</t>
+          <t>Option</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Resource</t>
+          <t>Option Text</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Correct Pos</t>
+          <t>Is Correct?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Scene Weight</t>
+          <t>Score</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>SG Role</t>
+          <t>SG Element</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Weight Rationale</t>
+          <t>Distractor Type</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Error Tag</t>
+          <t>Distractor Rationale</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>LRS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>SC06</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>OG0021_SC06_I</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Cause / low point</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>Milo cries; this begins the ending chain.</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>missed_cause_scene</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>SC07</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>OG0021_SC07_I</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Immediate result</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>The pond shines after the tear falls.</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>immediate_result_shift</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>SC08</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>OG0021_SC08_I</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Internal turn</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Milo realizes his color may be inside him.</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>realization_order</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>SC09</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>OG0021_SC09_I</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Final consequence</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>Milo's colors come back; final outcome receives high weight.</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>final_result_order</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D9" s="15">
-        <f>SUM(D5:D8)</f>
-        <v/>
+          <t>Student Weakness Signal</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>LRS sg_element</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>a yellow butterfly</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Character distractor</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Confuses the first character Milo meets with Milo himself.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Actor identity confusion</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>a little chameleon</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>SC01_ST01_N introduces Milo as a little chameleon.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>a red flower</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Object distractor</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Chooses a later object from the story as the main character.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Object/character confusion</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>a blue pond</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Place/object distractor</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Chooses a place or object rather than a character.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Place/character confusion</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q06_setting" | result.sg_element="setting" | result.score_raw=&lt;pts&gt;</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A10:I10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3118,7 +3179,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q07 — Synthesis MCQ | Main Idea / Whole Story Meaning</t>
+          <t>Q07 - Synthesis MCQ | Main Idea / Whole Story Meaning</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3238,7 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3187,12 +3248,12 @@
           <t>Colors keep you safe.</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="11" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3222,7 +3283,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3232,12 +3293,12 @@
           <t>Friends always help you.</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="12" t="n">
         <v>30</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3267,7 +3328,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3277,12 +3338,12 @@
           <t>Your color is inside you.</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3312,7 +3373,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3322,12 +3383,12 @@
           <t>The world has many colors.</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3357,7 +3418,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q07_synthesis" | result.sg_element="synthesis" | result.score_raw=&lt;pts&gt;</t>
         </is>
@@ -3394,7 +3455,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Story Grammar Scoring Model — v2</t>
+          <t>Story Grammar Scoring Model - v2</t>
         </is>
       </c>
     </row>
@@ -3436,248 +3497,248 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>setting_score</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Understands who/what the story begins with.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Initiating Event</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Q02</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event_score</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Understands what started the problem.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Attempt</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>attempt_score</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>weighted word sequence</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Understands what the character does to solve the problem.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>reaction_score</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Understands visible feeling/response.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Internal Response</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>internal_response_score</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Infers thoughts, motive, inner state.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Consequence</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
           <t>Q01</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>setting_score</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>weighted option score</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Understands the key place/background for the story action.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis 1</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>consequence_score</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>weighted scene position</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Understands result and event development.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>weighted average by story level</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Initiating Event</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Q02</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>initiating_event_score</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Synthesis</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Q07</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>synthesis_score</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>option score</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Understands what started the problem.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis 2</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Attempt</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>attempt_score</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>weighted word sequence</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Understands what the character does to solve the problem.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis 3</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>reaction_score</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Understands visible feeling/response.</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis 4</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Internal Response</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>internal_response_score</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Infers thoughts, motive, inner state.</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis 5</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Consequence</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Q06</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>consequence_score</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>weighted scene position</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Understands result and event development.</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis 6</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Synthesis</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Q07</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>synthesis_score</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Synthesizes whole-story meaning.</t>
@@ -3695,9 +3756,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Overall Reading Score = average(6 Story Grammar axes) × 0.8 + Synthesis × 0.2</t>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Overall Reading Score = average(6 Story Grammar axes) x 0.8 + Synthesis x 0.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update OG0021 v2 setting drag question
</commit_message>
<xml_diff>
--- a/v2/OG0021/OG0021_ReadingQuiz.xlsx
+++ b/v2/OG0021/OG0021_ReadingQuiz.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUIZ_LIST" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q01_CONSEQUENCE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q02_INIT_EVENT" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q03_ATTEMPT" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q04_REACTION" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q05_INTERNAL" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q06_SETTING" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q01_SETTING" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q02_CONSEQUENCE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q03_INIT_EVENT" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q04_ATTEMPT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q05_REACTION" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q06_INTERNAL" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q07_SYNTHESIS" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SG_SCORING" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LRS_MAPPING" sheetId="10" state="visible" r:id="rId10"/>
@@ -88,17 +88,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEECC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,20 +155,20 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -185,10 +185,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -563,8 +563,8 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -638,27 +638,27 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Story Scene Sequence</t>
+          <t>Setting Slot Drag</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Consequence</t>
+          <t>Setting</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Put the story scenes in order.</t>
+          <t>Choose the story start.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>SC01/02/03/06/09 images</t>
+          <t>Image-word cards</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>SC01 -&gt; SC02 -&gt; SC03 -&gt; SC06 -&gt; SC09</t>
+          <t>who=chameleon / where=forest / what=color</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -666,17 +666,17 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>consequence</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Weighted Position</t>
+          <t>Weighted Slot Match</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Q01_CONSEQUENCE</t>
+          <t>Q01_SETTING</t>
         </is>
       </c>
     </row>
@@ -688,27 +688,27 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Listening Scene Match</t>
+          <t>Story Scene Sequence</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Initiating Event</t>
+          <t>Consequence</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Listen. Which scene starts the problem?</t>
+          <t>Put the story scenes in order.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Audio + SC02/03/06/09</t>
+          <t>SC01/02/03/06/09 images</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Option A</t>
+          <t>SC01 -&gt; SC02 -&gt; SC03 -&gt; SC06 -&gt; SC09</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -716,17 +716,17 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>initiating_event</t>
+          <t>consequence</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Weighted MCQ</t>
+          <t>Weighted Position</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Q02_INIT_EVENT</t>
+          <t>Q02_CONSEQUENCE</t>
         </is>
       </c>
     </row>
@@ -738,27 +738,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Scene-Anchored Unscramble</t>
+          <t>Listening Scene Match</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Attempt</t>
+          <t>Initiating Event</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Put the story words in order.</t>
+          <t>Listen. Which scene starts the problem?</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>SC03 image</t>
+          <t>Audio + SC02/03/06/09</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Milo walks into the forest.</t>
+          <t>Option A</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -766,17 +766,17 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>attempt</t>
+          <t>initiating_event</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Weighted Unscramble</t>
+          <t>Weighted MCQ</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Q03_ATTEMPT</t>
+          <t>Q03_INIT_EVENT</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Feeling Match</t>
+          <t>Scene-Anchored Unscramble</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Reaction</t>
+          <t>Attempt</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>How does Milo feel here?</t>
+          <t>Put the story words in order.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>SC06 image</t>
+          <t>SC03 image</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Option B</t>
+          <t>Milo walks into the forest.</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -816,17 +816,17 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>reaction</t>
+          <t>attempt</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Weighted MCQ</t>
+          <t>Weighted Unscramble</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Q04_REACTION</t>
+          <t>Q04_ATTEMPT</t>
         </is>
       </c>
     </row>
@@ -838,17 +838,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Internal Response MCQ</t>
+          <t>Feeling Match</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Internal Response</t>
+          <t>Reaction</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>What is Milo thinking?</t>
+          <t>How does Milo feel here?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Option A</t>
+          <t>Option B</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -866,7 +866,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>internal_response</t>
+          <t>reaction</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Q05_INTERNAL</t>
+          <t>Q05_REACTION</t>
         </is>
       </c>
     </row>
@@ -888,27 +888,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Setting MCQ</t>
+          <t>Internal Response MCQ</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Internal Response</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Who is Milo at the beginning?</t>
+          <t>What is Milo thinking?</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SC06 image</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Option B</t>
+          <t>Option A</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>internal_response</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Q06_SETTING</t>
+          <t>Q06_INTERNAL</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Q01</t>
         </is>
@@ -1077,247 +1077,247 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>quiz_OG0021_v2_Q01_consequence</t>
+          <t>quiz_OG0021_v2_Q01_setting</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>setting</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>slot_values, component_scores</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Setting gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Q02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q02_consequence</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>consequence</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>partial</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>scene_order, component_scores</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Consequence gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Q02</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q02_initiating_event</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q03_initiating_event</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>initiating_event</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>true/false</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>option_selected, audio_src</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Initiating event gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q03_attempt</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q04_attempt</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>attempt</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>partial</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>word_order, word_scores</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Attempt/action gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q04_reaction</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q05_reaction</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>reaction</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>true/false</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>option_selected</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Reaction/emotion gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q05_internal_response</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q06_internal_response</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>internal_response</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>true/false</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>option_selected</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Inference gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Q06</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q06_setting</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>true/false</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>option_selected</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Setting gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Q07</t>
         </is>
@@ -1367,6 +1367,509 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Q01 - Setting Slot Drag | Story Grammar: Setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Question: Choose the story start.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Card Key</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Correct?</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Slot Weight</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Credit Rule</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Distractor Rationale</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>LRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>chameleon</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>chameleon</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Who?</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC01_I</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>100% if placed in Who</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Correct main character at the beginning.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>butterfly</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>butterfly</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Who?</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC03_I</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in Who</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Confuses first encountered character with Milo.</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>flower</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Who?</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC05_I</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in Who</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Chooses an object as the character.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Where?</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC03_I</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>100% if placed in Where</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Correct story place/background.</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>pond</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>pond</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Where?</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC06_I</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in Where</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Uses a later important place as the opening place.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Where?</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC10_I</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in Where</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Confuses ending place with opening/background.</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>What?</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC01_I</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>100% if placed in What</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Correct key thing related to the story start/problem.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>What?</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC06_I</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in What</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Uses a consequence clue as the starting clue.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>mirror</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>mirror</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>What?</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC10_I</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in What</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Uses an ending object as the key starting clue.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Scoring: full slot weight for exact target; 35% of slot weight for same-category distractor; 0 for wrong category.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A16:I16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1388,7 +1891,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q01 - Story Scene Sequence | Story Grammar: Consequence</t>
+          <t>Q02 - Story Scene Sequence | Story Grammar: Consequence</t>
         </is>
       </c>
     </row>
@@ -1480,30 +1983,30 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>SC02</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>OG0021_SC02_I</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Problem begins</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Milo wakes up gray; this is the key event that drives the rest of the story.</t>
+          <t>Milo wakes up gray; this key event drives the rest of the story.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1594,23 +2097,23 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>SC09</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>OG0021_SC09_I</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Final result</t>
         </is>
@@ -1632,12 +2135,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="10">
         <f>SUM(D5:D9)</f>
         <v/>
       </c>
@@ -1645,7 +2148,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q01_consequence" | result.sg_element="consequence" | result.score_raw=&lt;pts&gt;</t>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q02_consequence" | result.sg_element="consequence" | result.score_raw=&lt;pts&gt;</t>
         </is>
       </c>
     </row>
@@ -1659,7 +2162,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1682,7 +2185,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q02 - Listening Scene Match | Story Grammar: Initiating Event</t>
+          <t>Q03 - Listening Scene Match | Story Grammar: Initiating Event</t>
         </is>
       </c>
     </row>
@@ -1694,7 +2197,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Resource: Audio/OG0021_SC02_ST01_N_A.mp3</t>
         </is>
@@ -1748,7 +2251,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1758,12 +2261,12 @@
           <t>OG0021_SC02_I</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="6" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1793,7 +2296,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1803,12 +2306,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="7" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1930,7 +2433,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q02_init_event" | result.sg_element="initiating_event" | result.score_raw=&lt;pts&gt;</t>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q03_init_event" | result.sg_element="initiating_event" | result.score_raw=&lt;pts&gt;</t>
         </is>
       </c>
     </row>
@@ -1945,7 +2448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1968,7 +2471,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q03 - Scene-Anchored Unscramble | Story Grammar: Attempt</t>
+          <t>Q04 - Scene-Anchored Unscramble | Story Grammar: Attempt</t>
         </is>
       </c>
     </row>
@@ -1980,14 +2483,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Correct sentence from SC03_ST01_N: "Milo walks into the forest."</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Scrambled words: walks | forest. | Milo | the | into</t>
         </is>
@@ -2031,7 +2534,7 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Milo</t>
         </is>
@@ -2039,7 +2542,7 @@
       <c r="B7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
@@ -2063,7 +2566,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>walks</t>
         </is>
@@ -2071,7 +2574,7 @@
       <c r="B8" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Action verb</t>
         </is>
@@ -2095,7 +2598,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>into</t>
         </is>
@@ -2103,7 +2606,7 @@
       <c r="B9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Direction word</t>
         </is>
@@ -2127,7 +2630,7 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>the</t>
         </is>
@@ -2135,7 +2638,7 @@
       <c r="B10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
@@ -2159,7 +2662,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>forest.</t>
         </is>
@@ -2167,7 +2670,7 @@
       <c r="B11" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Place noun</t>
         </is>
@@ -2191,16 +2694,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="10">
         <f>SUM(D7:D11)</f>
         <v/>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="10">
         <f>SUM(F7:F11)</f>
         <v/>
       </c>
@@ -2280,7 +2783,7 @@
           <t>forest. into the walks Milo</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="7" t="n">
         <v>17</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2301,292 +2804,6 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:I4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Q04 - Feeling Match | Story Grammar: Reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Question: How does Milo feel here?</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Resource: OG0021_SC06_I.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Option Text</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Is Correct?</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>SG Element</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Distractor Type</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Distractor Rationale</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Student Weakness Signal</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>LRS sg_element</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Opposite emotion</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Confuses resolution emotion with sadness.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Temporal emotion confusion</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>SC06 shows crying and sadness.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>40</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Adjacent negative emotion</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Recognizes negative feeling but labels it too strongly.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Emotion differentiation</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Surprised</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Early-event emotion</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Confuses surprise with later sadness.</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Scene emotion mapping</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q04_reaction" | result.sg_element="reaction" | result.score_raw=&lt;pts&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A11:I11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2615,19 +2832,19 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q05 - Internal Response MCQ | Story Grammar: Internal Response</t>
+          <t>Q05 - Feeling Match | Story Grammar: Reaction</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: What is Milo thinking?</t>
+          <t>Question: How does Milo feel here?</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -2681,92 +2898,92 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Everyone has their own color.</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Opposite emotion</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Confuses resolution emotion with sadness.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Temporal emotion confusion</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D7" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Internal Response</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Uses the actual SC06 thought/sentence to infer Milo's inner state.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>SC06 shows crying and sadness.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>internal_response</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>I want to fly with the butterfly.</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Attempt detail</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Earlier action</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Confuses earlier butterfly scene with Milo's thought.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Thought/action confusion</t>
-        </is>
-      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>attempt</t>
+          <t>reaction</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2995,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>The pond is very blue.</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -2787,83 +3004,83 @@
         </is>
       </c>
       <c r="D8" s="12" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Surface observation</t>
+          <t>Reaction</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Visual detail</t>
+          <t>Adjacent negative emotion</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Sees visual detail but not internal state.</t>
+          <t>Recognizes negative feeling but labels it too strongly.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Surface-level inference</t>
+          <t>Emotion differentiation</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>internal_response</t>
+          <t>reaction</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>I do not need my color.</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
+          <t>Surprised</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
-        <v>0</v>
+      <c r="D9" s="7" t="n">
+        <v>20</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Opposite motive</t>
+          <t>Reaction</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Contradiction</t>
+          <t>Early-event emotion</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Contradicts Milo's motivation to find his color.</t>
+          <t>Confuses surprise with later sadness.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Motive inversion</t>
+          <t>Scene emotion mapping</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>internal_response</t>
+          <t>reaction</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q05_internal" | result.sg_element="internal_response" | result.score_raw=&lt;pts&gt;</t>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q05_reaction" | result.sg_element="reaction" | result.score_raw=&lt;pts&gt;</t>
         </is>
       </c>
     </row>
@@ -2884,7 +3101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2901,256 +3118,264 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q06 - Setting MCQ | Story Grammar: Setting</t>
+          <t>Q06 - Internal Response MCQ | Story Grammar: Internal Response</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Who is Milo at the beginning?</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+          <t>Question: What is Milo thinking?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Resource: OG0021_SC06_I.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Option Text</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Is Correct?</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>SG Element</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Distractor Type</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Distractor Rationale</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Student Weakness Signal</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>LRS sg_element</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>a yellow butterfly</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Everyone has their own color.</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Internal Response</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Uses the actual SC06 thought/sentence to infer Milo's inner state.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>internal_response</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>I want to fly with the butterfly.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Character distractor</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Confuses the first character Milo meets with Milo himself.</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Actor identity confusion</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>a little chameleon</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>SC01_ST01_N introduces Milo as a little chameleon.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Attempt detail</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Earlier action</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Confuses earlier butterfly scene with Milo's thought.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Thought/action confusion</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>attempt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>a red flower</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>The pond is very blue.</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Object distractor</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Chooses a later object from the story as the main character.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Object/character confusion</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="D8" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Surface observation</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Visual detail</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Sees visual detail but not internal state.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Surface-level inference</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>internal_response</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>a blue pond</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>I do not need my color.</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D9" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Place/object distractor</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Chooses a place or object rather than a character.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Place/character confusion</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q06_setting" | result.sg_element="setting" | result.score_raw=&lt;pts&gt;</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Opposite motive</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Contradiction</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Contradicts Milo's motivation to find his color.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Motive inversion</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>internal_response</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q06_internal" | result.sg_element="internal_response" | result.score_raw=&lt;pts&gt;</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A11:I11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3238,7 +3463,7 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3248,12 +3473,12 @@
           <t>Colors keep you safe.</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="7" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3328,7 +3553,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3338,12 +3563,12 @@
           <t>Your color is inside you.</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="6" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3373,7 +3598,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3383,12 +3608,12 @@
           <t>The world has many colors.</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="7" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3497,229 +3722,229 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Q01</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>setting_score</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>weighted slot match</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Builds who/where/what at the story start.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Initiating Event</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event_score</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Understands what started the problem.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Attempt</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>attempt_score</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>weighted word sequence</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Understands what the character does to solve the problem.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>reaction_score</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Understands visible feeling/response.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Internal Response</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>Q06</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>setting_score</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>internal_response_score</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>option score</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Understands who/what the story begins with.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Infers thoughts, motive, inner state.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Radar axis</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>weighted average by story level</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Initiating Event</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Consequence</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Q02</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>initiating_event_score</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Understands what started the problem.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>consequence_score</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>weighted scene position</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Understands result and event development.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Radar axis</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>weighted average by story level</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Attempt</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>attempt_score</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>weighted word sequence</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Understands what the character does to solve the problem.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>reaction_score</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Understands visible feeling/response.</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Internal Response</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>internal_response_score</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Infers thoughts, motive, inner state.</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Consequence</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Q01</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>consequence_score</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>weighted scene position</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Understands result and event development.</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Synthesis</t>
         </is>

</xml_diff>

<commit_message>
Refine OG0021 v2 setting layout and report cards
</commit_message>
<xml_diff>
--- a/v2/OG0021/OG0021_ReadingQuiz.xlsx
+++ b/v2/OG0021/OG0021_ReadingQuiz.xlsx
@@ -648,7 +648,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Choose the story start.</t>
+          <t>Choose Who, Where, and What.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1396,7 +1396,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Choose the story start.</t>
+          <t>Question: Choose Who, Where, and What.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorder OG0021 v2 sequence and setting items
</commit_message>
<xml_diff>
--- a/v2/OG0021/OG0021_ReadingQuiz.xlsx
+++ b/v2/OG0021/OG0021_ReadingQuiz.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUIZ_LIST" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q01_SETTING" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q02_CONSEQUENCE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q01_CONSEQUENCE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q02_SETTING" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q03_INIT_EVENT" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q04_ATTEMPT" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q05_REACTION" sheetId="6" state="visible" r:id="rId6"/>
@@ -88,17 +88,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEECC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,20 +155,20 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -185,10 +185,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -638,27 +638,27 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Setting Slot Drag</t>
+          <t>Story Scene Sequence</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Consequence</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Choose Who, Where, and What.</t>
+          <t>Put the story scenes in order.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Image-word cards</t>
+          <t>SC01/02/03/06/09 images</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>who=chameleon / where=forest / what=color</t>
+          <t>SC01 -&gt; SC02 -&gt; SC03 -&gt; SC06 -&gt; SC09</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -666,17 +666,17 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>setting</t>
+          <t>consequence</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Weighted Slot Match</t>
+          <t>Weighted Position</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Q01_SETTING</t>
+          <t>Q01_CONSEQUENCE</t>
         </is>
       </c>
     </row>
@@ -688,27 +688,27 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Story Scene Sequence</t>
+          <t>Setting Slot Drag</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Consequence</t>
+          <t>Setting</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Put the story scenes in order.</t>
+          <t>Look at the first scene. Fill in the boxes.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>SC01/02/03/06/09 images</t>
+          <t>SC01 image + word cards</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>SC01 -&gt; SC02 -&gt; SC03 -&gt; SC06 -&gt; SC09</t>
+          <t>who=chameleon / where=forest / at_first=loves changing colors</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -716,17 +716,17 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>consequence</t>
+          <t>setting</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Weighted Position</t>
+          <t>Weighted Slot Match</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Q02_CONSEQUENCE</t>
+          <t>Q02_SETTING</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Q01</t>
         </is>
@@ -1077,239 +1077,239 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>quiz_OG0021_v2_Q01_setting</t>
+          <t>quiz_OG0021_v2_Q01_consequence</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>consequence</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>scene_order, component_scores</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Consequence gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Q02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q02_setting</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>setting</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>partial</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>slot_values, component_scores</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Setting gap if &lt;70</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Q02</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q02_consequence</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q03_initiating_event</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>true/false</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>option_selected, audio_src</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Initiating event gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>answered</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q04_attempt</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>attempt</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>0-100</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>partial</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>scene_order, component_scores</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Consequence gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>word_order, word_scores</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Attempt/action gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q03_initiating_event</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>initiating_event</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q05_reaction</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>true/false</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>option_selected, audio_src</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Initiating event gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>option_selected</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Reaction/emotion gap if &lt;70</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>answered</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q04_attempt</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>attempt</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>quiz_OG0021_v2_Q06_internal_response</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>internal_response</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>0-100</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>partial</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>word_order, word_scores</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Attempt/action gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q05_reaction</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>true/false</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>option_selected</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Reaction/emotion gap if &lt;70</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Q06</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>answered</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>quiz_OG0021_v2_Q06_internal_response</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>internal_response</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>0-100</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>true/false</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>option_selected</t>
-        </is>
-      </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Inference gap if &lt;70</t>
@@ -1317,7 +1317,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Q07</t>
         </is>
@@ -1367,6 +1367,299 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Q01 - Story Scene Sequence | Story Grammar: Consequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Question: Put the story scenes in order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Scene</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Correct Pos</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Scene Weight</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>SG Role</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Weight Rationale</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Error Tag</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>LRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>SC01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>OG0021_SC01_I</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Opening state</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Shows Milo before the problem begins; useful context but lower weight than problem/result.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>missed_opening_state</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>consequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SC02</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OG0021_SC02_I</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Problem begins</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Milo wakes up gray; this key event drives the rest of the story.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>missed_problem_start</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SC03</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>OG0021_SC03_I</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Attempt begins</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Milo starts searching in the forest; a middle bridge scene.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>attempt_position_shift</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>attempt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>SC06</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>OG0021_SC06_I</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Low point / reaction</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Milo cries by the pond; shows the consequence before recovery.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>reaction_position_shift</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>reaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>SC09</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>OG0021_SC09_I</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Final result</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Milo's colors come back; final consequence gets high weight.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>missed_final_result</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>consequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D10" s="7">
+        <f>SUM(D5:D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q01_consequence" | result.sg_element="consequence" | result.score_raw=&lt;pts&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1389,14 +1682,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Q01 - Setting Slot Drag | Story Grammar: Setting</t>
+          <t>Q02 - Setting Slot Drag | Story Grammar: Setting</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Question: Choose Who, Where, and What.</t>
+          <t>Question: Look at the first scene. Fill in the boxes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Scene resource: OG0021_SC01_I.png</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1748,7 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>chameleon</t>
         </is>
@@ -1468,12 +1768,12 @@
           <t>OG0021_SC01_I</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="10" t="n">
         <v>2.5</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1493,7 +1793,7 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>butterfly</t>
         </is>
@@ -1513,12 +1813,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="11" t="n">
         <v>2.5</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1538,7 +1838,7 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>flower</t>
         </is>
@@ -1558,12 +1858,12 @@
           <t>OG0021_SC05_I</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="11" t="n">
         <v>2.5</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1583,7 +1883,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>forest</t>
         </is>
@@ -1603,12 +1903,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="10" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1628,7 +1928,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>pond</t>
         </is>
@@ -1648,12 +1948,12 @@
           <t>OG0021_SC06_I</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="11" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1673,7 +1973,7 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>home</t>
         </is>
@@ -1693,12 +1993,12 @@
           <t>OG0021_SC10_I</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="11" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1718,19 +2018,19 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>color</t>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>loves_colors</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>color</t>
+          <t>loves changing colors</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>What?</t>
+          <t>At first...</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1738,22 +2038,22 @@
           <t>OG0021_SC01_I</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="10" t="n">
         <v>1.5</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>100% if placed in What</t>
+          <t>100% if placed in At first</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Correct key thing related to the story start/problem.</t>
+          <t>Correct verb phrase from the opening state.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1763,87 +2063,87 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>tear</t>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>loses_color</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>tear</t>
+          <t>loses his color</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>What?</t>
+          <t>At first...</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
+          <t>OG0021_SC02_I</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in At first</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Uses the problem event as the opening state.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>cries_by_pond</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>cries by the pond</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>At first...</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
           <t>OG0021_SC06_I</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F13" s="11" t="n">
         <v>1.5</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>35% slot credit if placed in What</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Uses a consequence clue as the starting clue.</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>mirror</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>mirror</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>What?</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>OG0021_SC10_I</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>1.5</v>
-      </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>35% slot credit if placed in What</t>
+          <t>35% slot credit if placed in At first</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Uses an ending object as the key starting clue.</t>
+          <t>Uses a later reaction as the opening state.</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1860,303 +2160,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A16:I16"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Q02 - Story Scene Sequence | Story Grammar: Consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Question: Put the story scenes in order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Scene</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Resource</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Correct Pos</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Scene Weight</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>SG Role</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Weight Rationale</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Error Tag</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>LRS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>SC01</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>OG0021_SC01_I</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Opening state</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Shows Milo before the problem begins; useful context but lower weight than problem/result.</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>missed_opening_state</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>SC02</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>OG0021_SC02_I</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Problem begins</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Milo wakes up gray; this key event drives the rest of the story.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>missed_problem_start</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>initiating_event</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>SC03</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>OG0021_SC03_I</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Attempt begins</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Milo starts searching in the forest; a middle bridge scene.</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>attempt_position_shift</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>attempt</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>SC06</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>OG0021_SC06_I</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Low point / reaction</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Milo cries by the pond; shows the consequence before recovery.</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>reaction_position_shift</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>SC09</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>OG0021_SC09_I</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Final result</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Milo's colors come back; final consequence gets high weight.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>missed_final_result</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>consequence</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D10" s="10">
-        <f>SUM(D5:D9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>LRS xAPI: verb="answered" | object="quiz_OG0021_q02_consequence" | result.sg_element="consequence" | result.score_raw=&lt;pts&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2197,7 +2205,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Resource: Audio/OG0021_SC02_ST01_N_A.mp3</t>
         </is>
@@ -2251,7 +2259,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -2261,12 +2269,12 @@
           <t>OG0021_SC02_I</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2296,7 +2304,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2306,12 +2314,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2483,14 +2491,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Correct sentence from SC03_ST01_N: "Milo walks into the forest."</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Scrambled words: walks | forest. | Milo | the | into</t>
         </is>
@@ -2534,7 +2542,7 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Milo</t>
         </is>
@@ -2542,7 +2550,7 @@
       <c r="B7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
@@ -2566,7 +2574,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>walks</t>
         </is>
@@ -2574,7 +2582,7 @@
       <c r="B8" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Action verb</t>
         </is>
@@ -2598,7 +2606,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>into</t>
         </is>
@@ -2606,7 +2614,7 @@
       <c r="B9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Direction word</t>
         </is>
@@ -2630,7 +2638,7 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>the</t>
         </is>
@@ -2638,7 +2646,7 @@
       <c r="B10" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
@@ -2662,7 +2670,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>forest.</t>
         </is>
@@ -2670,7 +2678,7 @@
       <c r="B11" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Place noun</t>
         </is>
@@ -2694,16 +2702,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="7">
         <f>SUM(D7:D11)</f>
         <v/>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="7">
         <f>SUM(F7:F11)</f>
         <v/>
       </c>
@@ -2783,7 +2791,7 @@
           <t>forest. into the walks Milo</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="11" t="n">
         <v>17</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2844,7 +2852,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -2943,7 +2951,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2953,12 +2961,12 @@
           <t>Sad</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3033,7 +3041,7 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3043,12 +3051,12 @@
           <t>Surprised</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3130,7 +3138,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Resource: OG0021_SC06_I.png</t>
         </is>
@@ -3184,7 +3192,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3194,12 +3202,12 @@
           <t>Everyone has their own color.</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3229,7 +3237,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3239,12 +3247,12 @@
           <t>I want to fly with the butterfly.</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3463,7 +3471,7 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3473,12 +3481,12 @@
           <t>Colors keep you safe.</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="11" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3553,7 +3561,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3563,12 +3571,12 @@
           <t>Your color is inside you.</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="10" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3598,7 +3606,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3608,12 +3616,12 @@
           <t>The world has many colors.</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="11" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3722,229 +3730,229 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Q02</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>setting_score</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>weighted slot match</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Builds who/where/at-first information from the first scene.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Initiating Event</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Q03</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>initiating_event_score</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Understands what started the problem.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Attempt</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Q04</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>attempt_score</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>weighted word sequence</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Understands what the character does to solve the problem.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>reaction_score</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Understands visible feeling/response.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Internal Response</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>internal_response_score</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>option score</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Infers thoughts, motive, inner state.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Radar axis</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>weighted average by story level</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Consequence</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
           <t>Q01</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>setting_score</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>weighted slot match</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Builds who/where/what at the story start.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>consequence_score</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>weighted scene position</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Understands result and event development.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Radar axis</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>weighted average by story level</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Initiating Event</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Q03</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>initiating_event_score</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Understands what started the problem.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Attempt</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>attempt_score</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>weighted word sequence</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Understands what the character does to solve the problem.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Reaction</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Q05</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>reaction_score</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Understands visible feeling/response.</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Internal Response</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Q06</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>internal_response_score</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>option score</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Infers thoughts, motive, inner state.</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Consequence</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Q02</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>consequence_score</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>weighted scene position</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Understands result and event development.</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Radar axis</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>weighted average by story level</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Synthesis</t>
         </is>

</xml_diff>

<commit_message>
Polish OG0021 v2 layout and setting options
</commit_message>
<xml_diff>
--- a/v2/OG0021/OG0021_ReadingQuiz.xlsx
+++ b/v2/OG0021/OG0021_ReadingQuiz.xlsx
@@ -93,12 +93,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0070AD47"/>
+        <fgColor rgb="00FFEECC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEECC"/>
+        <fgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,10 +167,10 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -188,7 +188,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1665,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1750,40 +1750,40 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>chameleon</t>
+          <t>pond</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>chameleon</t>
+          <t>pond</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Who?</t>
+          <t>Where?</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>OG0021_SC01_I</t>
+          <t>OG0021_SC06_I</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F5" s="10" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>100% if placed in Who</t>
+          <t>35% slot credit if placed in Where</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Correct main character at the beginning.</t>
+          <t>Uses a later important place as the opening place.</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1795,12 +1795,12 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>butterfly</t>
+          <t>chameleon</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>butterfly</t>
+          <t>chameleon</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1810,12 +1810,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>OG0021_SC03_I</t>
+          <t>OG0021_SC01_I</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F6" s="11" t="n">
@@ -1823,12 +1823,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>35% slot credit if placed in Who</t>
+          <t>100% if placed in Who</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Confuses first encountered character with Milo.</t>
+          <t>Correct main character at the beginning.</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -1838,42 +1838,42 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>flower</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>loses_color</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>flower</t>
+          <t>loses his color</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Who?</t>
+          <t>At first...</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>OG0021_SC05_I</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
+          <t>OG0021_SC02_I</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F7" s="11" t="n">
-        <v>2.5</v>
+      <c r="F7" s="10" t="n">
+        <v>1.5</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>35% slot credit if placed in Who</t>
+          <t>35% slot credit if placed in At first</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Chooses an object as the character.</t>
+          <t>Uses the problem event as the opening state.</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>forest</t>
         </is>
@@ -1903,12 +1903,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1930,230 +1930,95 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>pond</t>
+          <t>loves_colors</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>pond</t>
+          <t>loves changing colors</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Where?</t>
+          <t>At first...</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>OG0021_SC06_I</t>
+          <t>OG0021_SC01_I</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>100% if placed in At first</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Correct verb phrase from the opening state.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>butterfly</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>butterfly</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Who?</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>OG0021_SC03_I</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F9" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>35% slot credit if placed in Where</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Uses a later important place as the opening place.</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="F10" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>35% slot credit if placed in Who</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Confuses first encountered character with Milo.</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Where?</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>OG0021_SC10_I</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>35% slot credit if placed in Where</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Confuses ending place with opening/background.</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>loves_colors</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>loves changing colors</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>At first...</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>OG0021_SC01_I</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>100% if placed in At first</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Correct verb phrase from the opening state.</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>loses_color</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>loses his color</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>At first...</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>OG0021_SC02_I</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>35% slot credit if placed in At first</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Uses the problem event as the opening state.</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>cries_by_pond</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>cries by the pond</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>At first...</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>OG0021_SC06_I</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>35% slot credit if placed in At first</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Uses a later reaction as the opening state.</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Scoring: full slot weight for exact target; 35% of slot weight for same-category distractor; 0 for wrong category.</t>
         </is>
@@ -2163,8 +2028,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A13:I13"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2259,7 +2124,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -2269,12 +2134,12 @@
           <t>OG0021_SC02_I</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2304,7 +2169,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2314,12 +2179,12 @@
           <t>OG0021_SC03_I</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="10" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2791,7 +2656,7 @@
           <t>forest. into the walks Milo</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="10" t="n">
         <v>17</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2951,7 +2816,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -2961,12 +2826,12 @@
           <t>Sad</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3041,7 +2906,7 @@
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3051,12 +2916,12 @@
           <t>Surprised</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="10" t="n">
         <v>20</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3192,7 +3057,7 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3202,12 +3067,12 @@
           <t>Everyone has their own color.</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <v>100</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -3237,7 +3102,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -3247,12 +3112,12 @@
           <t>I want to fly with the butterfly.</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="10" t="n">
         <v>20</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3471,7 +3336,7 @@
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -3481,12 +3346,12 @@
           <t>Colors keep you safe.</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="10" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3561,7 +3426,7 @@
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -3571,12 +3436,12 @@
           <t>Your color is inside you.</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -3606,7 +3471,7 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -3616,12 +3481,12 @@
           <t>The world has many colors.</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="10" t="n">
         <v>20</v>
       </c>
       <c r="E8" s="3" t="inlineStr">

</xml_diff>